<commit_message>
data added to servo offset
</commit_message>
<xml_diff>
--- a/Servo Offset.xlsx
+++ b/Servo Offset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ak574\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Github\AFIT_DigitalTwin_Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CF81D0E-7C3B-4AA6-ACE2-5E637F1D2BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50135592-9DB3-41CA-9070-951C197BBF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1842AE48-5C9A-47A1-9C64-879F0C5906AE}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11385" xr2:uid="{1842AE48-5C9A-47A1-9C64-879F0C5906AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>A0</t>
   </si>
@@ -48,6 +48,54 @@
   </si>
   <si>
     <t>Servo Offset:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/2'' scan : </t>
+  </si>
+  <si>
+    <t>All Sensor Value List : Small : 314 Large : 403</t>
+  </si>
+  <si>
+    <t>L Sensor Value List : Small : 360 Large : 403</t>
+  </si>
+  <si>
+    <t>R Sensor Value List : Small : 314 Large : 357</t>
+  </si>
+  <si>
+    <t>M Sensor Value List : Small : 348 Large : 386</t>
+  </si>
+  <si>
+    <t>1/4''</t>
+  </si>
+  <si>
+    <t>Color : 1/4</t>
+  </si>
+  <si>
+    <t>All Sensor Value List : Small : 230 Large : 396</t>
+  </si>
+  <si>
+    <t>L Sensor Value List : Small : 274 Large : 313</t>
+  </si>
+  <si>
+    <t>R Sensor Value List : Small : 230 Large : 277</t>
+  </si>
+  <si>
+    <t>M Sensor Value List : Small : 357 Large : 396</t>
+  </si>
+  <si>
+    <t>tl</t>
+  </si>
+  <si>
+    <t>All Sensor Value List : Small : 292 Large : 411</t>
+  </si>
+  <si>
+    <t>L Sensor Value List : Small : 292 Large : 341</t>
+  </si>
+  <si>
+    <t>R Sensor Value List : Small : 360 Large : 411</t>
+  </si>
+  <si>
+    <t>M Sensor Value List : Small : 334 Large : 377</t>
   </si>
 </sst>
 </file>
@@ -127,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -138,6 +186,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,8 +501,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{591BBB7C-F9CD-49EC-8B72-A9699E2FDAEE}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -505,6 +557,80 @@
         <v>0</v>
       </c>
       <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>